<commit_message>
feat: implement backend routing and frontend configuration management for DSCR parameters
</commit_message>
<xml_diff>
--- a/backend/guideline_type_parameters.xlsx
+++ b/backend/guideline_type_parameters.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LDNA40022\Lokesh\GuidelineIQ\backend\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AD042D8-8C38-4C05-B52B-2CB15B6301B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FC624F2-5FB0-41A7-B428-8AD2501826A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{8697C032-0460-4160-B668-D49F3090597F}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{8697C032-0460-4160-B668-D49F3090597F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="958" uniqueCount="237">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="910" uniqueCount="232">
   <si>
     <t>Parameters</t>
   </si>
@@ -687,85 +687,70 @@
     <t>Vesting &amp; Ownership</t>
   </si>
   <si>
-    <t>Borrower - DACA / ITIN</t>
-  </si>
-  <si>
-    <t>Borrower - Non-Permanent Resident Alien</t>
-  </si>
-  <si>
-    <t>Condo - Warrantable / Established Condos</t>
-  </si>
-  <si>
-    <t>Condo - Warrantable / Limited Review</t>
-  </si>
-  <si>
-    <t>Grantor Documentation for Entity Vesting</t>
-  </si>
-  <si>
-    <t>Housing History - Incomplete and Rent Free</t>
-  </si>
-  <si>
-    <t>Housing History Verification</t>
-  </si>
-  <si>
     <t>Lease and Occupancy Requirements</t>
   </si>
   <si>
     <t>Long Term Rentals</t>
   </si>
   <si>
-    <t>Vacant / Unleased Properties</t>
-  </si>
-  <si>
-    <t>Parameter</t>
-  </si>
-  <si>
-    <t>Loan Administration</t>
-  </si>
-  <si>
-    <t>Credit</t>
-  </si>
-  <si>
-    <t>DSCR Qualification</t>
-  </si>
-  <si>
-    <t>Income / DSCR</t>
-  </si>
-  <si>
-    <t>Financing Structure</t>
-  </si>
-  <si>
-    <t>Loan Limits / Eligibility</t>
-  </si>
-  <si>
-    <t>Product Features</t>
-  </si>
-  <si>
-    <t>Insurance</t>
-  </si>
-  <si>
-    <t>Property Cash Flow</t>
-  </si>
-  <si>
-    <t>Underwriting</t>
-  </si>
-  <si>
-    <t>Pricing</t>
-  </si>
-  <si>
-    <t>Transaction Requirements</t>
-  </si>
-  <si>
-    <t>Documentation</t>
-  </si>
-  <si>
-    <t>Geographic Restrictions</t>
-  </si>
-  <si>
-    <t>Title &amp; Legal</t>
-  </si>
-  <si>
-    <t>Income Documentation</t>
+    <t>Asset Depletion Income Calculation</t>
+  </si>
+  <si>
+    <t>Foreign National Visa Requirements</t>
+  </si>
+  <si>
+    <t>Non-Warrantable Condo Restrictions</t>
+  </si>
+  <si>
+    <t>Gift Fund Documentation</t>
+  </si>
+  <si>
+    <t>Employment Gap Requirements</t>
+  </si>
+  <si>
+    <t>Business Bank Statement Analysis</t>
+  </si>
+  <si>
+    <t>Deferred Student Loan Treatment</t>
+  </si>
+  <si>
+    <t>Recent Credit Inquiry Requirements</t>
+  </si>
+  <si>
+    <t>Escrow Waiver Eligibility</t>
+  </si>
+  <si>
+    <t>Property Insurance Requirements</t>
+  </si>
+  <si>
+    <t>LLC Operating Agreement Review</t>
+  </si>
+  <si>
+    <t>Short-Term Rental Eligibility</t>
+  </si>
+  <si>
+    <t>Bankruptcy Seasoning Requirements</t>
+  </si>
+  <si>
+    <t>Cash Reserve Calculation Method</t>
+  </si>
+  <si>
+    <t>Multiple Financed Properties Limit</t>
+  </si>
+  <si>
+    <t>Foreign Income Documentation</t>
+  </si>
+  <si>
+    <t>Bridge Loan Eligibility</t>
+  </si>
+  <si>
+    <t>Trust Vesting Requirements</t>
+  </si>
+  <si>
+    <t>Declining Market Restrictions</t>
+  </si>
+  <si>
+    <t>Self-Employed Borrower Analysis</t>
   </si>
 </sst>
 </file>
@@ -830,7 +815,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -853,22 +838,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -879,7 +853,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -895,14 +869,9 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3901,7 +3870,7 @@
     </row>
     <row r="188" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A188" s="6" t="s">
-        <v>217</v>
+        <v>210</v>
       </c>
       <c r="B188" s="4"/>
       <c r="C188" s="6" t="s">
@@ -3940,7 +3909,7 @@
     </row>
     <row r="191" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A191" s="6" t="s">
-        <v>218</v>
+        <v>211</v>
       </c>
       <c r="B191" s="4"/>
       <c r="C191" s="6" t="s">
@@ -4059,7 +4028,7 @@
       <c r="A200" s="6" t="s">
         <v>130</v>
       </c>
-      <c r="B200" s="10"/>
+      <c r="B200" s="4"/>
       <c r="C200" s="6" t="s">
         <v>23</v>
       </c>
@@ -4071,7 +4040,7 @@
       <c r="A201" s="6" t="s">
         <v>131</v>
       </c>
-      <c r="B201" s="10"/>
+      <c r="B201" s="4"/>
       <c r="C201" s="6" t="s">
         <v>23</v>
       </c>
@@ -4083,7 +4052,7 @@
       <c r="A202" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="B202" s="10"/>
+      <c r="B202" s="4"/>
       <c r="C202" s="6" t="s">
         <v>23</v>
       </c>
@@ -4095,7 +4064,7 @@
       <c r="A203" s="6" t="s">
         <v>134</v>
       </c>
-      <c r="B203" s="10"/>
+      <c r="B203" s="4"/>
       <c r="C203" s="6" t="s">
         <v>23</v>
       </c>
@@ -4107,7 +4076,7 @@
       <c r="A204" s="6" t="s">
         <v>201</v>
       </c>
-      <c r="B204" s="10"/>
+      <c r="B204" s="4"/>
       <c r="C204" s="6" t="s">
         <v>23</v>
       </c>
@@ -4119,7 +4088,7 @@
       <c r="A205" s="5" t="s">
         <v>137</v>
       </c>
-      <c r="B205" s="10"/>
+      <c r="B205" s="4"/>
       <c r="C205" s="6" t="s">
         <v>23</v>
       </c>
@@ -4131,7 +4100,7 @@
       <c r="A206" s="5" t="s">
         <v>202</v>
       </c>
-      <c r="B206" s="10"/>
+      <c r="B206" s="4"/>
       <c r="C206" s="6" t="s">
         <v>23</v>
       </c>
@@ -4143,7 +4112,7 @@
       <c r="A207" s="6" t="s">
         <v>203</v>
       </c>
-      <c r="B207" s="10"/>
+      <c r="B207" s="4"/>
       <c r="C207" s="6" t="s">
         <v>23</v>
       </c>
@@ -4155,7 +4124,7 @@
       <c r="A208" s="6" t="s">
         <v>204</v>
       </c>
-      <c r="B208" s="10"/>
+      <c r="B208" s="4"/>
       <c r="C208" s="6" t="s">
         <v>23</v>
       </c>
@@ -4167,7 +4136,7 @@
       <c r="A209" s="6" t="s">
         <v>145</v>
       </c>
-      <c r="B209" s="10"/>
+      <c r="B209" s="4"/>
       <c r="C209" s="6" t="s">
         <v>23</v>
       </c>
@@ -4179,7 +4148,7 @@
       <c r="A210" s="6" t="s">
         <v>205</v>
       </c>
-      <c r="B210" s="10"/>
+      <c r="B210" s="4"/>
       <c r="C210" s="6" t="s">
         <v>23</v>
       </c>
@@ -4191,7 +4160,7 @@
       <c r="A211" s="6" t="s">
         <v>153</v>
       </c>
-      <c r="B211" s="10"/>
+      <c r="B211" s="4"/>
       <c r="C211" s="6" t="s">
         <v>23</v>
       </c>
@@ -4203,7 +4172,7 @@
       <c r="A212" s="9" t="s">
         <v>191</v>
       </c>
-      <c r="B212" s="10"/>
+      <c r="B212" s="4"/>
       <c r="C212" s="6" t="s">
         <v>23</v>
       </c>
@@ -4215,7 +4184,7 @@
       <c r="A213" s="6" t="s">
         <v>159</v>
       </c>
-      <c r="B213" s="10"/>
+      <c r="B213" s="4"/>
       <c r="C213" s="6" t="s">
         <v>23</v>
       </c>
@@ -4227,7 +4196,7 @@
       <c r="A214" s="6" t="s">
         <v>206</v>
       </c>
-      <c r="B214" s="10"/>
+      <c r="B214" s="4"/>
       <c r="C214" s="6" t="s">
         <v>23</v>
       </c>
@@ -4239,7 +4208,7 @@
       <c r="A215" s="6" t="s">
         <v>207</v>
       </c>
-      <c r="B215" s="10"/>
+      <c r="B215" s="4"/>
       <c r="C215" s="6" t="s">
         <v>23</v>
       </c>
@@ -4248,10 +4217,10 @@
       </c>
     </row>
     <row r="216" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A216" s="11" t="s">
+      <c r="A216" s="10" t="s">
         <v>208</v>
       </c>
-      <c r="B216" s="10"/>
+      <c r="B216" s="4"/>
       <c r="C216" s="6" t="s">
         <v>23</v>
       </c>
@@ -4263,7 +4232,7 @@
       <c r="A217" s="6" t="s">
         <v>209</v>
       </c>
-      <c r="B217" s="10"/>
+      <c r="B217" s="4"/>
       <c r="C217" s="6" t="s">
         <v>23</v>
       </c>
@@ -4272,521 +4241,546 @@
       </c>
     </row>
     <row r="218" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A218" s="12"/>
-      <c r="C218" s="12"/>
-      <c r="D218" s="13"/>
-    </row>
-    <row r="241" spans="10:11" ht="29" x14ac:dyDescent="0.35">
-      <c r="J241" s="1" t="s">
+      <c r="A218" s="1"/>
+      <c r="B218" s="1"/>
+      <c r="C218" s="1"/>
+      <c r="D218" s="1"/>
+    </row>
+    <row r="219" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A219" s="2" t="s">
+        <v>212</v>
+      </c>
+      <c r="B219" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C219" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D219" s="2" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="220" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A220" s="2" t="s">
+        <v>213</v>
+      </c>
+      <c r="B220" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C220" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="D220" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="221" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A221" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="B221" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C221" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="D221" s="2" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="222" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A222" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="B222" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C222" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="D222" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="223" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A223" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="B223" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C223" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D223" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="224" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A224" s="2" t="s">
+        <v>217</v>
+      </c>
+      <c r="B224" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C224" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D224" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="225" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A225" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="B225" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C225" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D225" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="226" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A226" s="2" t="s">
+        <v>219</v>
+      </c>
+      <c r="B226" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C226" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D226" s="2" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="227" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A227" s="2" t="s">
         <v>220</v>
       </c>
-      <c r="K241" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="242" spans="10:11" ht="58" x14ac:dyDescent="0.35">
-      <c r="J242" s="2" t="s">
-        <v>167</v>
-      </c>
-      <c r="K242" s="2" t="s">
+      <c r="B227" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C227" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D227" s="2" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="228" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A228" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="B228" s="2" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="243" spans="10:11" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="J243" s="2" t="s">
-        <v>169</v>
-      </c>
-      <c r="K243" s="2" t="s">
+      <c r="C228" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="D228" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="229" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A229" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="B229" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C229" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="D229" s="2" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="230" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A230" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="B230" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="C230" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D230" s="2" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="231" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A231" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="B231" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C231" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D231" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="232" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A232" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="B232" s="2" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="244" spans="10:11" ht="87" x14ac:dyDescent="0.35">
-      <c r="J244" s="2" t="s">
-        <v>170</v>
-      </c>
-      <c r="K244" s="2" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="245" spans="10:11" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="J245" s="2" t="s">
-        <v>171</v>
-      </c>
-      <c r="K245" s="2" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="246" spans="10:11" ht="87" x14ac:dyDescent="0.35">
-      <c r="J246" s="2" t="s">
-        <v>172</v>
-      </c>
-      <c r="K246" s="2" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="247" spans="10:11" ht="29" x14ac:dyDescent="0.35">
-      <c r="J247" s="2" t="s">
-        <v>173</v>
-      </c>
-      <c r="K247" s="2" t="s">
+      <c r="C232" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D232" s="2" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="233" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A233" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="B233" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C233" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D233" s="2" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="234" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A234" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="B234" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C234" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="D234" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="235" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A235" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="B235" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C235" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="D235" s="2" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="236" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A236" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="B236" s="2" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="248" spans="10:11" ht="29" x14ac:dyDescent="0.35">
-      <c r="J248" s="2" t="s">
-        <v>174</v>
-      </c>
-      <c r="K248" s="2" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="249" spans="10:11" ht="87" x14ac:dyDescent="0.35">
-      <c r="J249" s="2" t="s">
-        <v>212</v>
-      </c>
-      <c r="K249" s="2" t="s">
+      <c r="C236" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="D236" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="237" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A237" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="B237" s="2" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="250" spans="10:11" ht="72.5" x14ac:dyDescent="0.35">
-      <c r="J250" s="2" t="s">
-        <v>213</v>
-      </c>
-      <c r="K250" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="251" spans="10:11" ht="101.5" x14ac:dyDescent="0.35">
-      <c r="J251" s="2" t="s">
-        <v>177</v>
-      </c>
-      <c r="K251" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="252" spans="10:11" ht="58" x14ac:dyDescent="0.35">
-      <c r="J252" s="2" t="s">
-        <v>178</v>
-      </c>
-      <c r="K252" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="253" spans="10:11" ht="58" x14ac:dyDescent="0.35">
-      <c r="J253" s="2" t="s">
-        <v>179</v>
-      </c>
-      <c r="K253" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="254" spans="10:11" ht="116" x14ac:dyDescent="0.35">
-      <c r="J254" s="2" t="s">
-        <v>180</v>
-      </c>
-      <c r="K254" s="2" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="255" spans="10:11" ht="29" x14ac:dyDescent="0.35">
-      <c r="J255" s="2" t="s">
-        <v>181</v>
-      </c>
-      <c r="K255" s="2" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="256" spans="10:11" ht="72.5" x14ac:dyDescent="0.35">
-      <c r="J256" s="2" t="s">
-        <v>182</v>
-      </c>
-      <c r="K256" s="2" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="257" spans="10:11" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="J257" s="2" t="s">
-        <v>210</v>
-      </c>
-      <c r="K257" s="2" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="258" spans="10:11" ht="58" x14ac:dyDescent="0.35">
-      <c r="J258" s="2" t="s">
-        <v>184</v>
-      </c>
-      <c r="K258" s="2" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="259" spans="10:11" ht="58" x14ac:dyDescent="0.35">
-      <c r="J259" s="2" t="s">
-        <v>185</v>
-      </c>
-      <c r="K259" s="2" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="260" spans="10:11" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="J260" s="2" t="s">
-        <v>186</v>
-      </c>
-      <c r="K260" s="2" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="261" spans="10:11" ht="72.5" x14ac:dyDescent="0.35">
-      <c r="J261" s="2" t="s">
-        <v>187</v>
-      </c>
-      <c r="K261" s="2" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="262" spans="10:11" ht="29" x14ac:dyDescent="0.35">
-      <c r="J262" s="2" t="s">
-        <v>188</v>
-      </c>
-      <c r="K262" s="2" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="263" spans="10:11" ht="72.5" x14ac:dyDescent="0.35">
-      <c r="J263" s="2" t="s">
-        <v>214</v>
-      </c>
-      <c r="K263" s="2" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="264" spans="10:11" ht="58" x14ac:dyDescent="0.35">
-      <c r="J264" s="2" t="s">
-        <v>190</v>
-      </c>
-      <c r="K264" s="2" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="265" spans="10:11" ht="116" x14ac:dyDescent="0.35">
-      <c r="J265" s="2" t="s">
-        <v>191</v>
-      </c>
-      <c r="K265" s="2" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="266" spans="10:11" ht="72.5" x14ac:dyDescent="0.35">
-      <c r="J266" s="2" t="s">
-        <v>215</v>
-      </c>
-      <c r="K266" s="2" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="267" spans="10:11" ht="58" x14ac:dyDescent="0.35">
-      <c r="J267" s="2" t="s">
-        <v>216</v>
-      </c>
-      <c r="K267" s="2" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="268" spans="10:11" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="J268" s="2" t="s">
-        <v>194</v>
-      </c>
-      <c r="K268" s="2" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="269" spans="10:11" ht="101.5" x14ac:dyDescent="0.35">
-      <c r="J269" s="2" t="s">
-        <v>195</v>
-      </c>
-      <c r="K269" s="2" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="270" spans="10:11" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="J270" s="2" t="s">
-        <v>196</v>
-      </c>
-      <c r="K270" s="2" t="s">
-        <v>226</v>
-      </c>
-    </row>
-    <row r="271" spans="10:11" ht="87" x14ac:dyDescent="0.35">
-      <c r="J271" s="2" t="s">
-        <v>197</v>
-      </c>
-      <c r="K271" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="272" spans="10:11" ht="87" x14ac:dyDescent="0.35">
-      <c r="J272" s="2" t="s">
-        <v>211</v>
-      </c>
-      <c r="K272" s="2" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="273" spans="10:11" ht="29" x14ac:dyDescent="0.35">
-      <c r="J273" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="K273" s="2" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="274" spans="10:11" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="J274" s="2" t="s">
-        <v>200</v>
-      </c>
-      <c r="K274" s="2" t="s">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="275" spans="10:11" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="J275" s="2" t="s">
-        <v>201</v>
-      </c>
-      <c r="K275" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="276" spans="10:11" ht="58" x14ac:dyDescent="0.35">
-      <c r="J276" s="2" t="s">
-        <v>202</v>
-      </c>
-      <c r="K276" s="2" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="277" spans="10:11" ht="58" x14ac:dyDescent="0.35">
-      <c r="J277" s="2" t="s">
-        <v>203</v>
-      </c>
-      <c r="K277" s="2" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="278" spans="10:11" ht="29" x14ac:dyDescent="0.35">
-      <c r="J278" s="2" t="s">
-        <v>140</v>
-      </c>
-      <c r="K278" s="2" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="279" spans="10:11" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="J279" s="2" t="s">
-        <v>205</v>
-      </c>
-      <c r="K279" s="2" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="280" spans="10:11" ht="58" x14ac:dyDescent="0.35">
-      <c r="J280" s="2" t="s">
-        <v>206</v>
-      </c>
-      <c r="K280" s="2" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="281" spans="10:11" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="J281" s="2" t="s">
-        <v>207</v>
-      </c>
-      <c r="K281" s="2" t="s">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="282" spans="10:11" ht="58" x14ac:dyDescent="0.35">
-      <c r="J282" s="2" t="s">
-        <v>219</v>
-      </c>
-      <c r="K282" s="2" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="283" spans="10:11" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="J283" s="2" t="s">
-        <v>209</v>
-      </c>
-      <c r="K283" s="2" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="284" spans="10:11" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="J284" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="K284" s="2" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="285" spans="10:11" ht="29" x14ac:dyDescent="0.35">
-      <c r="J285" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="K285" s="2" t="s">
+      <c r="C237" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D237" s="2" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="238" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A238" s="2" t="s">
         <v>231</v>
       </c>
-    </row>
-    <row r="286" spans="10:11" ht="29" x14ac:dyDescent="0.35">
-      <c r="J286" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="K286" s="2" t="s">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="287" spans="10:11" ht="58" x14ac:dyDescent="0.35">
-      <c r="J287" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="K287" s="2" t="s">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="288" spans="10:11" ht="87" x14ac:dyDescent="0.35">
-      <c r="J288" s="2" t="s">
-        <v>217</v>
-      </c>
-      <c r="K288" s="2" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="289" spans="10:11" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="J289" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="K289" s="2" t="s">
-        <v>226</v>
-      </c>
-    </row>
-    <row r="290" spans="10:11" ht="29" x14ac:dyDescent="0.35">
-      <c r="J290" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="K290" s="2" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="291" spans="10:11" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="J291" s="2" t="s">
-        <v>218</v>
-      </c>
-      <c r="K291" s="2" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="292" spans="10:11" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="J292" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="K292" s="2" t="s">
-        <v>226</v>
-      </c>
-    </row>
-    <row r="293" spans="10:11" ht="58" x14ac:dyDescent="0.35">
-      <c r="J293" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="K293" s="2" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="294" spans="10:11" ht="58" x14ac:dyDescent="0.35">
-      <c r="J294" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="K294" s="2" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="295" spans="10:11" ht="29" x14ac:dyDescent="0.35">
-      <c r="J295" s="2" t="s">
-        <v>127</v>
-      </c>
-      <c r="K295" s="2" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="296" spans="10:11" ht="29" x14ac:dyDescent="0.35">
-      <c r="J296" s="2" t="s">
-        <v>130</v>
-      </c>
-      <c r="K296" s="2" t="s">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="297" spans="10:11" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="J297" s="2" t="s">
-        <v>131</v>
-      </c>
-      <c r="K297" s="2" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="298" spans="10:11" ht="58" x14ac:dyDescent="0.35">
-      <c r="J298" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="K298" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="299" spans="10:11" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="J299" s="2" t="s">
-        <v>134</v>
-      </c>
-      <c r="K299" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="300" spans="10:11" ht="58" x14ac:dyDescent="0.35">
-      <c r="J300" s="2" t="s">
-        <v>137</v>
-      </c>
-      <c r="K300" s="2" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="301" spans="10:11" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="J301" s="2" t="s">
-        <v>145</v>
-      </c>
-      <c r="K301" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="302" spans="10:11" ht="58" x14ac:dyDescent="0.35">
-      <c r="J302" s="2" t="s">
-        <v>153</v>
-      </c>
-      <c r="K302" s="2" t="s">
-        <v>234</v>
-      </c>
-    </row>
-    <row r="303" spans="10:11" ht="72.5" x14ac:dyDescent="0.35">
-      <c r="J303" s="2" t="s">
-        <v>159</v>
-      </c>
-      <c r="K303" s="2" t="s">
-        <v>235</v>
-      </c>
-    </row>
-    <row r="304" spans="10:11" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="J304" s="2" t="s">
-        <v>166</v>
-      </c>
-      <c r="K304" s="2" t="s">
-        <v>236</v>
-      </c>
+      <c r="B238" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C238" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D238" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="241" spans="10:11" x14ac:dyDescent="0.35">
+      <c r="J241" s="1"/>
+      <c r="K241" s="1"/>
+    </row>
+    <row r="242" spans="10:11" x14ac:dyDescent="0.35">
+      <c r="J242" s="2"/>
+      <c r="K242" s="2"/>
+    </row>
+    <row r="243" spans="10:11" x14ac:dyDescent="0.35">
+      <c r="J243" s="2"/>
+      <c r="K243" s="2"/>
+    </row>
+    <row r="244" spans="10:11" x14ac:dyDescent="0.35">
+      <c r="J244" s="2"/>
+      <c r="K244" s="2"/>
+    </row>
+    <row r="245" spans="10:11" x14ac:dyDescent="0.35">
+      <c r="J245" s="2"/>
+      <c r="K245" s="2"/>
+    </row>
+    <row r="246" spans="10:11" x14ac:dyDescent="0.35">
+      <c r="J246" s="2"/>
+      <c r="K246" s="2"/>
+    </row>
+    <row r="247" spans="10:11" x14ac:dyDescent="0.35">
+      <c r="J247" s="2"/>
+      <c r="K247" s="2"/>
+    </row>
+    <row r="248" spans="10:11" x14ac:dyDescent="0.35">
+      <c r="J248" s="2"/>
+      <c r="K248" s="2"/>
+    </row>
+    <row r="249" spans="10:11" x14ac:dyDescent="0.35">
+      <c r="J249" s="2"/>
+      <c r="K249" s="2"/>
+    </row>
+    <row r="250" spans="10:11" x14ac:dyDescent="0.35">
+      <c r="J250" s="2"/>
+      <c r="K250" s="2"/>
+    </row>
+    <row r="251" spans="10:11" x14ac:dyDescent="0.35">
+      <c r="J251" s="2"/>
+      <c r="K251" s="2"/>
+    </row>
+    <row r="252" spans="10:11" x14ac:dyDescent="0.35">
+      <c r="J252" s="2"/>
+      <c r="K252" s="2"/>
+    </row>
+    <row r="253" spans="10:11" x14ac:dyDescent="0.35">
+      <c r="J253" s="2"/>
+      <c r="K253" s="2"/>
+    </row>
+    <row r="254" spans="10:11" x14ac:dyDescent="0.35">
+      <c r="J254" s="2"/>
+      <c r="K254" s="2"/>
+    </row>
+    <row r="255" spans="10:11" x14ac:dyDescent="0.35">
+      <c r="J255" s="2"/>
+      <c r="K255" s="2"/>
+    </row>
+    <row r="256" spans="10:11" x14ac:dyDescent="0.35">
+      <c r="J256" s="2"/>
+      <c r="K256" s="2"/>
+    </row>
+    <row r="257" spans="10:11" x14ac:dyDescent="0.35">
+      <c r="J257" s="2"/>
+      <c r="K257" s="2"/>
+    </row>
+    <row r="258" spans="10:11" x14ac:dyDescent="0.35">
+      <c r="J258" s="2"/>
+      <c r="K258" s="2"/>
+    </row>
+    <row r="259" spans="10:11" x14ac:dyDescent="0.35">
+      <c r="J259" s="2"/>
+      <c r="K259" s="2"/>
+    </row>
+    <row r="260" spans="10:11" x14ac:dyDescent="0.35">
+      <c r="J260" s="2"/>
+      <c r="K260" s="2"/>
+    </row>
+    <row r="261" spans="10:11" x14ac:dyDescent="0.35">
+      <c r="J261" s="2"/>
+      <c r="K261" s="2"/>
+    </row>
+    <row r="262" spans="10:11" x14ac:dyDescent="0.35">
+      <c r="J262" s="2"/>
+      <c r="K262" s="2"/>
+    </row>
+    <row r="263" spans="10:11" x14ac:dyDescent="0.35">
+      <c r="J263" s="2"/>
+      <c r="K263" s="2"/>
+    </row>
+    <row r="264" spans="10:11" x14ac:dyDescent="0.35">
+      <c r="J264" s="2"/>
+      <c r="K264" s="2"/>
+    </row>
+    <row r="265" spans="10:11" x14ac:dyDescent="0.35">
+      <c r="J265" s="2"/>
+      <c r="K265" s="2"/>
+    </row>
+    <row r="266" spans="10:11" x14ac:dyDescent="0.35">
+      <c r="J266" s="2"/>
+      <c r="K266" s="2"/>
+    </row>
+    <row r="267" spans="10:11" x14ac:dyDescent="0.35">
+      <c r="J267" s="2"/>
+      <c r="K267" s="2"/>
+    </row>
+    <row r="268" spans="10:11" x14ac:dyDescent="0.35">
+      <c r="J268" s="2"/>
+      <c r="K268" s="2"/>
+    </row>
+    <row r="269" spans="10:11" x14ac:dyDescent="0.35">
+      <c r="J269" s="2"/>
+      <c r="K269" s="2"/>
+    </row>
+    <row r="270" spans="10:11" x14ac:dyDescent="0.35">
+      <c r="J270" s="2"/>
+      <c r="K270" s="2"/>
+    </row>
+    <row r="271" spans="10:11" x14ac:dyDescent="0.35">
+      <c r="J271" s="2"/>
+      <c r="K271" s="2"/>
+    </row>
+    <row r="272" spans="10:11" x14ac:dyDescent="0.35">
+      <c r="J272" s="2"/>
+      <c r="K272" s="2"/>
+    </row>
+    <row r="273" spans="10:11" x14ac:dyDescent="0.35">
+      <c r="J273" s="2"/>
+      <c r="K273" s="2"/>
+    </row>
+    <row r="274" spans="10:11" x14ac:dyDescent="0.35">
+      <c r="J274" s="2"/>
+      <c r="K274" s="2"/>
+    </row>
+    <row r="275" spans="10:11" x14ac:dyDescent="0.35">
+      <c r="J275" s="2"/>
+      <c r="K275" s="2"/>
+    </row>
+    <row r="276" spans="10:11" x14ac:dyDescent="0.35">
+      <c r="J276" s="2"/>
+      <c r="K276" s="2"/>
+    </row>
+    <row r="277" spans="10:11" x14ac:dyDescent="0.35">
+      <c r="J277" s="2"/>
+      <c r="K277" s="2"/>
+    </row>
+    <row r="278" spans="10:11" x14ac:dyDescent="0.35">
+      <c r="J278" s="2"/>
+      <c r="K278" s="2"/>
+    </row>
+    <row r="279" spans="10:11" x14ac:dyDescent="0.35">
+      <c r="J279" s="2"/>
+      <c r="K279" s="2"/>
+    </row>
+    <row r="280" spans="10:11" x14ac:dyDescent="0.35">
+      <c r="J280" s="2"/>
+      <c r="K280" s="2"/>
+    </row>
+    <row r="281" spans="10:11" x14ac:dyDescent="0.35">
+      <c r="J281" s="2"/>
+      <c r="K281" s="2"/>
+    </row>
+    <row r="282" spans="10:11" x14ac:dyDescent="0.35">
+      <c r="J282" s="2"/>
+      <c r="K282" s="2"/>
+    </row>
+    <row r="283" spans="10:11" x14ac:dyDescent="0.35">
+      <c r="J283" s="2"/>
+      <c r="K283" s="2"/>
+    </row>
+    <row r="284" spans="10:11" x14ac:dyDescent="0.35">
+      <c r="J284" s="2"/>
+      <c r="K284" s="2"/>
+    </row>
+    <row r="285" spans="10:11" x14ac:dyDescent="0.35">
+      <c r="J285" s="2"/>
+      <c r="K285" s="2"/>
+    </row>
+    <row r="286" spans="10:11" x14ac:dyDescent="0.35">
+      <c r="J286" s="2"/>
+      <c r="K286" s="2"/>
+    </row>
+    <row r="287" spans="10:11" x14ac:dyDescent="0.35">
+      <c r="J287" s="2"/>
+      <c r="K287" s="2"/>
+    </row>
+    <row r="288" spans="10:11" x14ac:dyDescent="0.35">
+      <c r="J288" s="2"/>
+      <c r="K288" s="2"/>
+    </row>
+    <row r="289" spans="10:11" x14ac:dyDescent="0.35">
+      <c r="J289" s="2"/>
+      <c r="K289" s="2"/>
+    </row>
+    <row r="290" spans="10:11" x14ac:dyDescent="0.35">
+      <c r="J290" s="2"/>
+      <c r="K290" s="2"/>
+    </row>
+    <row r="291" spans="10:11" x14ac:dyDescent="0.35">
+      <c r="J291" s="2"/>
+      <c r="K291" s="2"/>
+    </row>
+    <row r="292" spans="10:11" x14ac:dyDescent="0.35">
+      <c r="J292" s="2"/>
+      <c r="K292" s="2"/>
+    </row>
+    <row r="293" spans="10:11" x14ac:dyDescent="0.35">
+      <c r="J293" s="2"/>
+      <c r="K293" s="2"/>
+    </row>
+    <row r="294" spans="10:11" x14ac:dyDescent="0.35">
+      <c r="J294" s="2"/>
+      <c r="K294" s="2"/>
+    </row>
+    <row r="295" spans="10:11" x14ac:dyDescent="0.35">
+      <c r="J295" s="2"/>
+      <c r="K295" s="2"/>
+    </row>
+    <row r="296" spans="10:11" x14ac:dyDescent="0.35">
+      <c r="J296" s="2"/>
+      <c r="K296" s="2"/>
+    </row>
+    <row r="297" spans="10:11" x14ac:dyDescent="0.35">
+      <c r="J297" s="2"/>
+      <c r="K297" s="2"/>
+    </row>
+    <row r="298" spans="10:11" x14ac:dyDescent="0.35">
+      <c r="J298" s="2"/>
+      <c r="K298" s="2"/>
+    </row>
+    <row r="299" spans="10:11" x14ac:dyDescent="0.35">
+      <c r="J299" s="2"/>
+      <c r="K299" s="2"/>
+    </row>
+    <row r="300" spans="10:11" x14ac:dyDescent="0.35">
+      <c r="J300" s="2"/>
+      <c r="K300" s="2"/>
+    </row>
+    <row r="301" spans="10:11" x14ac:dyDescent="0.35">
+      <c r="J301" s="2"/>
+      <c r="K301" s="2"/>
+    </row>
+    <row r="302" spans="10:11" x14ac:dyDescent="0.35">
+      <c r="J302" s="2"/>
+      <c r="K302" s="2"/>
+    </row>
+    <row r="303" spans="10:11" x14ac:dyDescent="0.35">
+      <c r="J303" s="2"/>
+      <c r="K303" s="2"/>
+    </row>
+    <row r="304" spans="10:11" x14ac:dyDescent="0.35">
+      <c r="J304" s="2"/>
+      <c r="K304" s="2"/>
     </row>
   </sheetData>
   <dataValidations count="1">
@@ -4799,6 +4793,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100763FE7442E5DD84E9ED81A67B08353FE" ma:contentTypeVersion="13" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="d5442ab2fb4245c444331d98c5b124c5">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns3="03c0eb20-715c-4472-b31d-a609615d6f17" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="7a03aacb61114f2d9c840004b805593e" ns1:_="" ns3:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -5003,15 +5006,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -5023,6 +5017,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{85BE1DFB-7D3F-4386-BDD2-7B855B7EFB24}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B3ED73A6-4C88-4FC5-9BE1-3CB2EE0765FC}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -5037,14 +5039,6 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{85BE1DFB-7D3F-4386-BDD2-7B855B7EFB24}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
feat: implement DSCR parameter management API and configuration UI
</commit_message>
<xml_diff>
--- a/backend/guideline_type_parameters.xlsx
+++ b/backend/guideline_type_parameters.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LDNA40022\Lokesh\GuidelineIQ\backend\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FC624F2-5FB0-41A7-B428-8AD2501826A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B080F3C0-0B61-4BE2-A3D2-CE6F029EE143}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{8697C032-0460-4160-B668-D49F3090597F}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{8697C032-0460-4160-B668-D49F3090597F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="910" uniqueCount="232">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="867" uniqueCount="212">
   <si>
     <t>Parameters</t>
   </si>
@@ -54,9 +54,6 @@
   </si>
   <si>
     <t>Income Doc Type</t>
-  </si>
-  <si>
-    <t>Full &amp; Alt</t>
   </si>
   <si>
     <t>2-1 Buydown</t>
@@ -693,64 +690,7 @@
     <t>Long Term Rentals</t>
   </si>
   <si>
-    <t>Asset Depletion Income Calculation</t>
-  </si>
-  <si>
-    <t>Foreign National Visa Requirements</t>
-  </si>
-  <si>
-    <t>Non-Warrantable Condo Restrictions</t>
-  </si>
-  <si>
-    <t>Gift Fund Documentation</t>
-  </si>
-  <si>
-    <t>Employment Gap Requirements</t>
-  </si>
-  <si>
-    <t>Business Bank Statement Analysis</t>
-  </si>
-  <si>
-    <t>Deferred Student Loan Treatment</t>
-  </si>
-  <si>
-    <t>Recent Credit Inquiry Requirements</t>
-  </si>
-  <si>
-    <t>Escrow Waiver Eligibility</t>
-  </si>
-  <si>
-    <t>Property Insurance Requirements</t>
-  </si>
-  <si>
-    <t>LLC Operating Agreement Review</t>
-  </si>
-  <si>
-    <t>Short-Term Rental Eligibility</t>
-  </si>
-  <si>
-    <t>Bankruptcy Seasoning Requirements</t>
-  </si>
-  <si>
-    <t>Cash Reserve Calculation Method</t>
-  </si>
-  <si>
-    <t>Multiple Financed Properties Limit</t>
-  </si>
-  <si>
-    <t>Foreign Income Documentation</t>
-  </si>
-  <si>
-    <t>Bridge Loan Eligibility</t>
-  </si>
-  <si>
-    <t>Trust Vesting Requirements</t>
-  </si>
-  <si>
-    <t>Declining Market Restrictions</t>
-  </si>
-  <si>
-    <t>Self-Employed Borrower Analysis</t>
+    <t>Full, Alt</t>
   </si>
 </sst>
 </file>
@@ -1240,236 +1180,236 @@
         <v>5</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" s="5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B3" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="5" t="s">
-        <v>9</v>
-      </c>
       <c r="D3" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="6" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B4" s="6" t="s">
         <v>4</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B5" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="5" t="s">
-        <v>13</v>
-      </c>
       <c r="C5" s="5" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" s="6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" s="5" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B8" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="B8" s="5" t="s">
-        <v>17</v>
-      </c>
       <c r="C8" s="5" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" s="5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="B10" s="5" t="s">
         <v>19</v>
-      </c>
-      <c r="B10" s="5" t="s">
-        <v>20</v>
       </c>
       <c r="C10" s="5" t="s">
         <v>5</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="B11" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="B11" s="6" t="s">
-        <v>22</v>
-      </c>
       <c r="C11" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" s="5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" s="5" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B14" s="5" t="s">
         <v>4</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" s="5" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B15" s="5" t="s">
         <v>4</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="B16" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="B16" s="5" t="s">
+      <c r="C16" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="C16" s="5" t="s">
-        <v>30</v>
-      </c>
       <c r="D16" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="B17" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="C17" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="B17" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="C17" s="5" t="s">
-        <v>32</v>
-      </c>
       <c r="D17" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" s="5" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19" s="5" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B19" s="5" t="s">
         <v>4</v>
@@ -1478,1076 +1418,1076 @@
         <v>5</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20" s="5" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C20" s="5" t="s">
         <v>5</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A21" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C21" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="B21" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="C21" s="5" t="s">
-        <v>37</v>
-      </c>
       <c r="D21" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A22" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="B22" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C22" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="B22" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="C22" s="5" t="s">
-        <v>39</v>
-      </c>
       <c r="D22" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A23" s="5" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A24" s="6" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A25" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="B25" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="B25" s="5" t="s">
-        <v>43</v>
-      </c>
       <c r="C25" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A26" s="6" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B26" s="6" t="s">
         <v>4</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A27" s="5" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A28" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="B28" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="C28" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="B28" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="C28" s="5" t="s">
-        <v>47</v>
-      </c>
       <c r="D28" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A29" s="5" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A30" s="6" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B30" s="6" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A31" s="5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A32" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B32" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="C32" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="B32" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="C32" s="5" t="s">
-        <v>52</v>
-      </c>
       <c r="D32" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A33" s="5" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D33" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A34" s="6" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B34" s="6" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D34" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A35" s="5" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A36" s="5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C36" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A37" s="6" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B37" s="6" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C37" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D37" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A38" s="5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D38" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A39" s="5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C39" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D39" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A40" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B40" s="5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D40" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A41" s="5" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B41" s="5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C41" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D41" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A42" s="5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B42" s="5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C42" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D42" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A43" s="6" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B43" s="6" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C43" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D43" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A44" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="B44" s="5" t="s">
         <v>64</v>
-      </c>
-      <c r="B44" s="5" t="s">
-        <v>65</v>
       </c>
       <c r="C44" s="5" t="s">
         <v>5</v>
       </c>
       <c r="D44" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A45" s="5" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B45" s="5" t="s">
         <v>4</v>
       </c>
       <c r="C45" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D45" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A46" s="5" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B46" s="5" t="s">
         <v>4</v>
       </c>
       <c r="C46" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D46" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A47" s="6" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B47" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C47" s="5" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D47" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A48" s="5" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B48" s="5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C48" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D48" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A49" s="6" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B49" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C49" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D49" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A50" s="6" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B50" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C50" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D50" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A51" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="B51" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="C51" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="B51" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="C51" s="5" t="s">
-        <v>73</v>
-      </c>
       <c r="D51" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A52" s="5" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B52" s="5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C52" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D52" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A53" s="6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B53" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C53" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D53" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A54" s="5" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B54" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C54" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D54" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A55" s="5" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B55" s="5" t="s">
         <v>4</v>
       </c>
       <c r="C55" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D55" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A56" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="B56" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="C56" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="B56" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="C56" s="6" t="s">
-        <v>79</v>
-      </c>
       <c r="D56" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A57" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B57" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C57" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D57" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A58" s="6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B58" s="6" t="s">
         <v>4</v>
       </c>
       <c r="C58" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D58" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A59" s="5" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B59" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C59" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D59" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A60" s="5" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B60" s="5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C60" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D60" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A61" s="5" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B61" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C61" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D61" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A62" s="5" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B62" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C62" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D62" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A63" s="6" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B63" s="6" t="s">
         <v>4</v>
       </c>
       <c r="C63" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D63" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A64" s="6" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B64" s="6" t="s">
         <v>4</v>
       </c>
       <c r="C64" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D64" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A65" s="5" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B65" s="5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C65" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D65" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A66" s="6" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B66" s="6" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C66" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D66" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A67" s="6" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B67" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C67" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D67" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A68" s="5" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B68" s="5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C68" s="5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D68" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A69" s="6" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B69" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C69" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D69" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A70" s="5" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B70" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C70" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D70" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A71" s="5" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B71" s="5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C71" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D71" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A72" s="6" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B72" s="6" t="s">
         <v>4</v>
       </c>
       <c r="C72" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D72" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A73" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B73" s="5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C73" s="5" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D73" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A74" s="6" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B74" s="6" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C74" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D74" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A75" s="5" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B75" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C75" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D75" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A76" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="B76" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="B76" s="5" t="s">
-        <v>100</v>
-      </c>
       <c r="C76" s="5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D76" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A77" s="5" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B77" s="5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C77" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D77" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A78" s="6" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B78" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C78" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D78" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A79" s="5" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B79" s="5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C79" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D79" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A80" s="5" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B80" s="5" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C80" s="5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D80" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A81" s="6" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B81" s="5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C81" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D81" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A82" s="5" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B82" s="5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C82" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D82" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A83" s="5" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B83" s="5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C83" s="5" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D83" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A84" s="5" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B84" s="5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C84" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D84" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A85" s="6" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B85" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C85" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D85" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A86" s="5" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B86" s="5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C86" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D86" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A87" s="6" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B87" s="6" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C87" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D87" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A88" s="5" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B88" s="5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C88" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D88" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A89" s="5" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B89" s="5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C89" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D89" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A90" s="5" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B90" s="5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C90" s="5" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D90" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A91" s="6" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B91" s="6" t="s">
         <v>4</v>
       </c>
       <c r="C91" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D91" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A92" s="5" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B92" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C92" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D92" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A93" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="B93" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C93" s="5" t="s">
         <v>116</v>
       </c>
-      <c r="B93" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="C93" s="5" t="s">
-        <v>117</v>
-      </c>
       <c r="D93" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A94" s="5" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B94" s="5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C94" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D94" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A95" s="6" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B95" s="6" t="s">
         <v>4</v>
       </c>
       <c r="C95" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D95" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A96" s="5" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B96" s="5" t="s">
         <v>4</v>
@@ -2556,26 +2496,26 @@
         <v>5</v>
       </c>
       <c r="D96" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A97" s="5" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B97" s="5" t="s">
         <v>4</v>
       </c>
       <c r="C97" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D97" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A98" s="5" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B98" s="5" t="s">
         <v>4</v>
@@ -2584,558 +2524,558 @@
         <v>5</v>
       </c>
       <c r="D98" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A99" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B99" s="6" t="s">
         <v>4</v>
       </c>
       <c r="C99" s="5" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D99" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A100" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="B100" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="C100" s="5" t="s">
         <v>124</v>
       </c>
-      <c r="B100" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="C100" s="5" t="s">
-        <v>125</v>
-      </c>
       <c r="D100" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A101" s="6" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B101" s="6" t="s">
         <v>4</v>
       </c>
       <c r="C101" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D101" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A102" s="5" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B102" s="5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C102" s="5" t="s">
         <v>5</v>
       </c>
       <c r="D102" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A103" s="5" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B103" s="5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C103" s="5" t="s">
         <v>5</v>
       </c>
       <c r="D103" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A104" s="6" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B104" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C104" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D104" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A105" s="5" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B105" s="5" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C105" s="5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D105" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A106" s="5" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B106" s="5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C106" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D106" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A107" s="5" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B107" s="5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C107" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D107" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A108" s="5" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B108" s="5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C108" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D108" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A109" s="5" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B109" s="5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C109" s="5" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D109" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A110" s="6" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B110" s="6" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C110" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D110" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A111" s="5" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B111" s="5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C111" s="5" t="s">
         <v>5</v>
       </c>
       <c r="D111" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A112" s="5" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B112" s="5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C112" s="5" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D112" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="113" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A113" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="B113" s="5" t="s">
         <v>138</v>
       </c>
-      <c r="B113" s="5" t="s">
-        <v>139</v>
-      </c>
       <c r="C113" s="5" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D113" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A114" s="5" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B114" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C114" s="5" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D114" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A115" s="5" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B115" s="5" t="s">
         <v>4</v>
       </c>
       <c r="C115" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D115" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A116" s="6" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B116" s="6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C116" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D116" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A117" s="6" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B117" s="6" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C117" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D117" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="118" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A118" s="6" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B118" s="6" t="s">
         <v>4</v>
       </c>
       <c r="C118" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D118" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="119" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A119" s="6" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B119" s="6" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C119" s="5" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D119" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="120" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A120" s="5" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B120" s="5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C120" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D120" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A121" s="5" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B121" s="5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C121" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D121" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A122" s="6" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B122" s="6" t="s">
         <v>4</v>
       </c>
       <c r="C122" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D122" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="123" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A123" s="5" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B123" s="5" t="s">
         <v>4</v>
       </c>
       <c r="C123" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D123" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="124" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A124" s="6" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B124" s="6" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C124" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D124" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="125" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A125" s="6" t="s">
+        <v>150</v>
+      </c>
+      <c r="B125" s="6" t="s">
         <v>151</v>
       </c>
-      <c r="B125" s="6" t="s">
-        <v>152</v>
-      </c>
       <c r="C125" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D125" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="126" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A126" s="6" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B126" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C126" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D126" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="127" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A127" s="5" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B127" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C127" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D127" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="128" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A128" s="5" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B128" s="5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C128" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D128" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="129" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A129" s="5" t="s">
+        <v>155</v>
+      </c>
+      <c r="B129" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C129" s="5" t="s">
         <v>156</v>
       </c>
-      <c r="B129" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="C129" s="5" t="s">
-        <v>157</v>
-      </c>
       <c r="D129" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="130" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A130" s="5" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B130" s="5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C130" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D130" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="131" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A131" s="6" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B131" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C131" s="5" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D131" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="132" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A132" s="5" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B132" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C132" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D132" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="133" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A133" s="6" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B133" s="6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C133" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D133" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="134" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A134" s="5" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B134" s="5" t="s">
         <v>4</v>
       </c>
       <c r="C134" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D134" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="135" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A135" s="5" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B135" s="5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C135" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D135" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="136" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A136" s="6" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B136" s="6" t="s">
         <v>4</v>
       </c>
       <c r="C136" s="5" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D136" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="137" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A137" s="6" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B137" s="6" t="s">
         <v>4</v>
       </c>
       <c r="C137" s="5" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D137" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="138" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A138" s="5" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B138" s="5" t="s">
         <v>4</v>
@@ -3144,1387 +3084,1301 @@
         <v>5</v>
       </c>
       <c r="D138" s="4" t="s">
-        <v>6</v>
+        <v>211</v>
       </c>
     </row>
     <row r="139" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A139" s="6" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B139" s="5" t="s">
-        <v>13</v>
+        <v>28</v>
       </c>
       <c r="C139" s="5" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D139" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E139" s="2"/>
     </row>
     <row r="140" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A140" s="6" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B140" s="6" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="C140" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D140" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E140" s="2"/>
     </row>
     <row r="141" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A141" s="5" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B141" s="6" t="s">
-        <v>22</v>
+        <v>7</v>
       </c>
       <c r="C141" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D141" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E141" s="2"/>
     </row>
     <row r="142" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A142" s="5" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B142" s="6" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="C142" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D142" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E142" s="2"/>
     </row>
     <row r="143" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A143" s="6" t="s">
-        <v>172</v>
-      </c>
-      <c r="B143" s="6" t="s">
-        <v>8</v>
+        <v>171</v>
+      </c>
+      <c r="B143" s="5" t="s">
+        <v>7</v>
       </c>
       <c r="C143" s="6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D143" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E143" s="2"/>
     </row>
     <row r="144" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A144" s="5" t="s">
-        <v>173</v>
-      </c>
-      <c r="B144" s="5" t="s">
+        <v>172</v>
+      </c>
+      <c r="B144" s="6" t="s">
+        <v>167</v>
+      </c>
+      <c r="C144" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="C144" s="5" t="s">
-        <v>30</v>
-      </c>
       <c r="D144" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E144" s="2"/>
     </row>
     <row r="145" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A145" s="6" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B145" s="6" t="s">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="C145" s="6" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D145" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E145" s="2"/>
     </row>
     <row r="146" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A146" s="6" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B146" s="6" t="s">
-        <v>13</v>
+        <v>167</v>
       </c>
       <c r="C146" s="6" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D146" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E146" s="2"/>
     </row>
     <row r="147" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A147" s="6" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B147" s="6" t="s">
-        <v>13</v>
+        <v>42</v>
       </c>
       <c r="C147" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D147" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E147" s="2"/>
     </row>
     <row r="148" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A148" s="6" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B148" s="6" t="s">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="C148" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D148" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E148" s="2"/>
     </row>
     <row r="149" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A149" s="6" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B149" s="6" t="s">
-        <v>22</v>
+        <v>7</v>
       </c>
       <c r="C149" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D149" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E149" s="2"/>
     </row>
     <row r="150" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A150" s="6" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B150" s="6" t="s">
-        <v>13</v>
+        <v>28</v>
       </c>
       <c r="C150" s="6" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D150" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E150" s="2"/>
     </row>
     <row r="151" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A151" s="6" t="s">
-        <v>180</v>
-      </c>
-      <c r="B151" s="6" t="s">
-        <v>8</v>
+        <v>179</v>
+      </c>
+      <c r="B151" s="5" t="s">
+        <v>12</v>
       </c>
       <c r="C151" s="6" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D151" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E151" s="2"/>
     </row>
     <row r="152" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A152" s="6" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B152" s="6" t="s">
-        <v>43</v>
+        <v>21</v>
       </c>
       <c r="C152" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D152" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E152" s="2"/>
     </row>
     <row r="153" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A153" s="6" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B153" s="6" t="s">
-        <v>43</v>
+        <v>21</v>
       </c>
       <c r="C153" s="6" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D153" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E153" s="2"/>
     </row>
     <row r="154" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A154" s="5" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="B154" s="6" t="s">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="C154" s="6" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D154" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E154" s="2"/>
     </row>
     <row r="155" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A155" s="6" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B155" s="6" t="s">
-        <v>168</v>
+        <v>7</v>
       </c>
       <c r="C155" s="6" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D155" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E155" s="2"/>
     </row>
     <row r="156" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A156" s="6" t="s">
-        <v>185</v>
-      </c>
-      <c r="B156" s="6" t="s">
-        <v>29</v>
+        <v>184</v>
+      </c>
+      <c r="B156" s="5" t="s">
+        <v>28</v>
       </c>
       <c r="C156" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D156" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E156" s="2"/>
     </row>
     <row r="157" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A157" s="6" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B157" s="6" t="s">
-        <v>29</v>
+        <v>7</v>
       </c>
       <c r="C157" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D157" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E157" s="2"/>
     </row>
     <row r="158" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A158" s="6" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B158" s="6" t="s">
-        <v>29</v>
+        <v>12</v>
       </c>
       <c r="C158" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D158" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E158" s="2"/>
     </row>
     <row r="159" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A159" s="6" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B159" s="6" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="C159" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D159" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E159" s="2"/>
     </row>
     <row r="160" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A160" s="6" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B160" s="6" t="s">
-        <v>29</v>
+        <v>12</v>
       </c>
       <c r="C160" s="6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D160" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E160" s="2"/>
     </row>
     <row r="161" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A161" s="5" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B161" s="6" t="s">
-        <v>168</v>
+        <v>21</v>
       </c>
       <c r="C161" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D161" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E161" s="2"/>
     </row>
     <row r="162" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A162" s="5" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B162" s="6" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="C162" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D162" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E162" s="2"/>
     </row>
     <row r="163" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A163" s="6" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B163" s="6" t="s">
-        <v>43</v>
+        <v>7</v>
       </c>
       <c r="C163" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D163" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E163" s="2"/>
     </row>
     <row r="164" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A164" s="5" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B164" s="6" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C164" s="6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D164" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E164" s="2"/>
     </row>
     <row r="165" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A165" s="6" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B165" s="6" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C165" s="6" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D165" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E165" s="2"/>
     </row>
     <row r="166" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A166" s="5" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B166" s="6" t="s">
-        <v>43</v>
+        <v>28</v>
       </c>
       <c r="C166" s="6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D166" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E166" s="2"/>
     </row>
     <row r="167" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A167" s="6" t="s">
-        <v>196</v>
-      </c>
-      <c r="B167" s="5" t="s">
-        <v>65</v>
+        <v>195</v>
+      </c>
+      <c r="B167" s="6" t="s">
+        <v>167</v>
       </c>
       <c r="C167" s="5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D167" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E167" s="2"/>
     </row>
     <row r="168" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A168" s="6" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B168" s="6" t="s">
-        <v>8</v>
+        <v>28</v>
       </c>
       <c r="C168" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D168" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E168" s="2"/>
     </row>
     <row r="169" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A169" s="6" t="s">
-        <v>198</v>
-      </c>
-      <c r="B169" s="5" t="s">
-        <v>29</v>
+        <v>197</v>
+      </c>
+      <c r="B169" s="6" t="s">
+        <v>28</v>
       </c>
       <c r="C169" s="5" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D169" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E169" s="2"/>
     </row>
     <row r="170" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A170" s="6" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B170" s="6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C170" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D170" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E170" s="2"/>
     </row>
     <row r="171" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A171" s="6" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B171" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C171" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="C171" s="6" t="s">
-        <v>9</v>
-      </c>
       <c r="D171" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E171" s="2"/>
     </row>
     <row r="172" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A172" s="6" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B172" s="6" t="s">
-        <v>13</v>
+        <v>28</v>
       </c>
       <c r="C172" s="6" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D172" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E172" s="2"/>
     </row>
     <row r="173" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A173" s="5" t="s">
-        <v>202</v>
-      </c>
-      <c r="B173" s="5" t="s">
-        <v>8</v>
+        <v>201</v>
+      </c>
+      <c r="B173" s="6" t="s">
+        <v>167</v>
       </c>
       <c r="C173" s="5" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D173" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E173" s="2"/>
     </row>
     <row r="174" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A174" s="6" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="B174" s="6" t="s">
-        <v>168</v>
+        <v>7</v>
       </c>
       <c r="C174" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D174" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E174" s="2"/>
     </row>
     <row r="175" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A175" s="6" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B175" s="6" t="s">
-        <v>22</v>
+        <v>42</v>
       </c>
       <c r="C175" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D175" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E175" s="2"/>
     </row>
     <row r="176" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A176" s="6" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="B176" s="6" t="s">
-        <v>168</v>
+        <v>42</v>
       </c>
       <c r="C176" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D176" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E176" s="2"/>
     </row>
     <row r="177" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A177" s="6" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B177" s="6" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C177" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D177" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E177" s="2"/>
     </row>
     <row r="178" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A178" s="6" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B178" s="6" t="s">
-        <v>8</v>
+        <v>42</v>
       </c>
       <c r="C178" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D178" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E178" s="2"/>
     </row>
     <row r="179" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A179" s="7" t="s">
-        <v>208</v>
-      </c>
-      <c r="B179" s="6" t="s">
-        <v>8</v>
+        <v>207</v>
+      </c>
+      <c r="B179" s="5" t="s">
+        <v>64</v>
       </c>
       <c r="C179" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D179" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E179" s="2"/>
     </row>
     <row r="180" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A180" s="6" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="B180" s="6" t="s">
-        <v>29</v>
+        <v>7</v>
       </c>
       <c r="C180" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D180" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E180" s="2"/>
     </row>
     <row r="181" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A181" s="8" t="s">
-        <v>192</v>
-      </c>
-      <c r="B181" s="4"/>
+        <v>191</v>
+      </c>
+      <c r="B181" s="6" t="s">
+        <v>42</v>
+      </c>
       <c r="C181" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D181" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E181" s="2"/>
     </row>
     <row r="182" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A182" s="9" t="s">
-        <v>193</v>
-      </c>
-      <c r="B182" s="4"/>
+        <v>192</v>
+      </c>
+      <c r="B182" s="6" t="s">
+        <v>42</v>
+      </c>
       <c r="C182" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D182" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E182" s="2"/>
     </row>
     <row r="183" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A183" s="9" t="s">
-        <v>195</v>
-      </c>
-      <c r="B183" s="4"/>
+        <v>194</v>
+      </c>
+      <c r="B183" s="5" t="s">
+        <v>64</v>
+      </c>
       <c r="C183" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D183" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E183" s="2"/>
     </row>
     <row r="184" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A184" s="5" t="s">
-        <v>88</v>
-      </c>
-      <c r="B184" s="4"/>
+        <v>87</v>
+      </c>
+      <c r="B184" s="6" t="s">
+        <v>7</v>
+      </c>
       <c r="C184" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D184" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E184" s="2"/>
     </row>
     <row r="185" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A185" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="B185" s="4"/>
+        <v>89</v>
+      </c>
+      <c r="B185" s="6" t="s">
+        <v>42</v>
+      </c>
       <c r="C185" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D185" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E185" s="2"/>
     </row>
     <row r="186" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A186" s="5" t="s">
-        <v>91</v>
-      </c>
-      <c r="B186" s="4"/>
+        <v>90</v>
+      </c>
+      <c r="B186" s="5" t="s">
+        <v>28</v>
+      </c>
       <c r="C186" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D186" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E186" s="2"/>
     </row>
     <row r="187" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A187" s="6" t="s">
-        <v>92</v>
-      </c>
-      <c r="B187" s="4"/>
+        <v>91</v>
+      </c>
+      <c r="B187" s="6" t="s">
+        <v>7</v>
+      </c>
       <c r="C187" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D187" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E187" s="2"/>
     </row>
     <row r="188" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A188" s="6" t="s">
-        <v>210</v>
-      </c>
-      <c r="B188" s="4"/>
+        <v>209</v>
+      </c>
+      <c r="B188" s="6" t="s">
+        <v>12</v>
+      </c>
       <c r="C188" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D188" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E188" s="2"/>
     </row>
     <row r="189" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A189" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="B189" s="4"/>
+        <v>98</v>
+      </c>
+      <c r="B189" s="6" t="s">
+        <v>12</v>
+      </c>
       <c r="C189" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D189" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E189" s="2"/>
     </row>
     <row r="190" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A190" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="B190" s="4"/>
+        <v>38</v>
+      </c>
+      <c r="B190" s="6" t="s">
+        <v>12</v>
+      </c>
       <c r="C190" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D190" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E190" s="2"/>
     </row>
     <row r="191" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A191" s="6" t="s">
-        <v>211</v>
-      </c>
-      <c r="B191" s="4"/>
+        <v>210</v>
+      </c>
+      <c r="B191" s="6" t="s">
+        <v>21</v>
+      </c>
       <c r="C191" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D191" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E191" s="2"/>
     </row>
     <row r="192" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A192" s="8" t="s">
-        <v>196</v>
-      </c>
-      <c r="B192" s="4"/>
+        <v>195</v>
+      </c>
+      <c r="B192" s="6" t="s">
+        <v>12</v>
+      </c>
       <c r="C192" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D192" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E192" s="2"/>
     </row>
     <row r="193" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A193" s="6" t="s">
-        <v>197</v>
-      </c>
-      <c r="B193" s="4"/>
+        <v>196</v>
+      </c>
+      <c r="B193" s="6" t="s">
+        <v>7</v>
+      </c>
       <c r="C193" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D193" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E193" s="2"/>
     </row>
     <row r="194" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A194" s="6" t="s">
-        <v>104</v>
-      </c>
-      <c r="B194" s="4"/>
+        <v>103</v>
+      </c>
+      <c r="B194" s="6" t="s">
+        <v>42</v>
+      </c>
       <c r="C194" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D194" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E194" s="2"/>
     </row>
     <row r="195" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A195" s="6" t="s">
-        <v>108</v>
-      </c>
-      <c r="B195" s="4"/>
+        <v>107</v>
+      </c>
+      <c r="B195" s="6" t="s">
+        <v>42</v>
+      </c>
       <c r="C195" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D195" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E195" s="2"/>
     </row>
     <row r="196" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A196" s="6" t="s">
-        <v>124</v>
-      </c>
-      <c r="B196" s="4"/>
+        <v>123</v>
+      </c>
+      <c r="B196" s="6" t="s">
+        <v>28</v>
+      </c>
       <c r="C196" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D196" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E196" s="2"/>
     </row>
     <row r="197" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A197" s="6" t="s">
-        <v>199</v>
-      </c>
-      <c r="B197" s="4"/>
+        <v>198</v>
+      </c>
+      <c r="B197" s="6" t="s">
+        <v>167</v>
+      </c>
       <c r="C197" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D197" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E197" s="2"/>
     </row>
     <row r="198" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A198" s="6" t="s">
-        <v>127</v>
-      </c>
-      <c r="B198" s="4"/>
+        <v>126</v>
+      </c>
+      <c r="B198" s="6" t="s">
+        <v>28</v>
+      </c>
       <c r="C198" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D198" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E198" s="2"/>
     </row>
     <row r="199" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A199" s="6" t="s">
-        <v>200</v>
-      </c>
-      <c r="B199" s="4"/>
+        <v>199</v>
+      </c>
+      <c r="B199" s="6" t="s">
+        <v>28</v>
+      </c>
       <c r="C199" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D199" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E199" s="2"/>
     </row>
     <row r="200" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A200" s="6" t="s">
-        <v>130</v>
-      </c>
-      <c r="B200" s="4"/>
+        <v>129</v>
+      </c>
+      <c r="B200" s="6" t="s">
+        <v>28</v>
+      </c>
       <c r="C200" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D200" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="201" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A201" s="6" t="s">
-        <v>131</v>
-      </c>
-      <c r="B201" s="4"/>
+        <v>130</v>
+      </c>
+      <c r="B201" s="6" t="s">
+        <v>21</v>
+      </c>
       <c r="C201" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D201" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="202" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A202" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="B202" s="4"/>
+        <v>13</v>
+      </c>
+      <c r="B202" s="6" t="s">
+        <v>28</v>
+      </c>
       <c r="C202" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D202" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="203" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A203" s="6" t="s">
-        <v>134</v>
-      </c>
-      <c r="B203" s="4"/>
+        <v>133</v>
+      </c>
+      <c r="B203" s="6" t="s">
+        <v>167</v>
+      </c>
       <c r="C203" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D203" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="204" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A204" s="6" t="s">
-        <v>201</v>
-      </c>
-      <c r="B204" s="4"/>
+        <v>200</v>
+      </c>
+      <c r="B204" s="6" t="s">
+        <v>7</v>
+      </c>
       <c r="C204" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D204" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="205" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A205" s="5" t="s">
-        <v>137</v>
-      </c>
-      <c r="B205" s="4"/>
+        <v>136</v>
+      </c>
+      <c r="B205" s="6" t="s">
+        <v>42</v>
+      </c>
       <c r="C205" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D205" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="206" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A206" s="5" t="s">
-        <v>202</v>
-      </c>
-      <c r="B206" s="4"/>
+        <v>201</v>
+      </c>
+      <c r="B206" s="6" t="s">
+        <v>42</v>
+      </c>
       <c r="C206" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D206" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="207" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A207" s="6" t="s">
-        <v>203</v>
-      </c>
-      <c r="B207" s="4"/>
+        <v>202</v>
+      </c>
+      <c r="B207" s="6" t="s">
+        <v>42</v>
+      </c>
       <c r="C207" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D207" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="208" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A208" s="6" t="s">
-        <v>204</v>
-      </c>
-      <c r="B208" s="4"/>
+        <v>203</v>
+      </c>
+      <c r="B208" s="6" t="s">
+        <v>42</v>
+      </c>
       <c r="C208" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D208" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="209" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A209" s="6" t="s">
-        <v>145</v>
-      </c>
-      <c r="B209" s="4"/>
+        <v>144</v>
+      </c>
+      <c r="B209" s="5" t="s">
+        <v>64</v>
+      </c>
       <c r="C209" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D209" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="210" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A210" s="6" t="s">
-        <v>205</v>
-      </c>
-      <c r="B210" s="4"/>
+        <v>204</v>
+      </c>
+      <c r="B210" s="6" t="s">
+        <v>7</v>
+      </c>
       <c r="C210" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D210" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="211" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A211" s="6" t="s">
-        <v>153</v>
-      </c>
-      <c r="B211" s="4"/>
+        <v>152</v>
+      </c>
+      <c r="B211" s="6" t="s">
+        <v>42</v>
+      </c>
       <c r="C211" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D211" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="212" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A212" s="9" t="s">
-        <v>191</v>
-      </c>
-      <c r="B212" s="4"/>
+        <v>190</v>
+      </c>
+      <c r="B212" s="6" t="s">
+        <v>42</v>
+      </c>
       <c r="C212" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D212" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="213" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A213" s="6" t="s">
-        <v>159</v>
-      </c>
-      <c r="B213" s="4"/>
+        <v>158</v>
+      </c>
+      <c r="B213" s="5" t="s">
+        <v>64</v>
+      </c>
       <c r="C213" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D213" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="214" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A214" s="6" t="s">
-        <v>206</v>
-      </c>
-      <c r="B214" s="4"/>
+        <v>205</v>
+      </c>
+      <c r="B214" s="6" t="s">
+        <v>7</v>
+      </c>
       <c r="C214" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D214" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="215" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A215" s="6" t="s">
-        <v>207</v>
-      </c>
-      <c r="B215" s="4"/>
+        <v>206</v>
+      </c>
+      <c r="B215" s="6" t="s">
+        <v>42</v>
+      </c>
       <c r="C215" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D215" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="216" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A216" s="10" t="s">
-        <v>208</v>
-      </c>
-      <c r="B216" s="4"/>
+        <v>207</v>
+      </c>
+      <c r="B216" s="6" t="s">
+        <v>42</v>
+      </c>
       <c r="C216" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D216" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="217" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A217" s="6" t="s">
-        <v>209</v>
-      </c>
-      <c r="B217" s="4"/>
+        <v>208</v>
+      </c>
+      <c r="B217" s="5" t="s">
+        <v>64</v>
+      </c>
       <c r="C217" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D217" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="218" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A218" s="1"/>
-      <c r="B218" s="1"/>
+      <c r="B218" s="6"/>
       <c r="C218" s="1"/>
       <c r="D218" s="1"/>
     </row>
-    <row r="219" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A219" s="2" t="s">
-        <v>212</v>
-      </c>
-      <c r="B219" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C219" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D219" s="2" t="s">
-        <v>168</v>
-      </c>
-    </row>
     <row r="220" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A220" s="2" t="s">
-        <v>213</v>
-      </c>
-      <c r="B220" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C220" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="D220" s="2" t="s">
-        <v>6</v>
-      </c>
+      <c r="A220" s="2"/>
+      <c r="B220" s="2"/>
+      <c r="C220" s="2"/>
+      <c r="D220" s="2"/>
     </row>
     <row r="221" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A221" s="2" t="s">
-        <v>214</v>
-      </c>
-      <c r="B221" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C221" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="D221" s="2" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="222" spans="1:4" ht="29" x14ac:dyDescent="0.35">
-      <c r="A222" s="2" t="s">
-        <v>215</v>
-      </c>
-      <c r="B222" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="C222" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="D222" s="2" t="s">
-        <v>6</v>
-      </c>
+      <c r="A221" s="2"/>
+      <c r="B221" s="2"/>
+      <c r="C221" s="2"/>
+      <c r="D221" s="2"/>
+    </row>
+    <row r="222" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A222" s="2"/>
+      <c r="B222" s="2"/>
+      <c r="C222" s="2"/>
+      <c r="D222" s="2"/>
     </row>
     <row r="223" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A223" s="2" t="s">
-        <v>216</v>
-      </c>
-      <c r="B223" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C223" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D223" s="2" t="s">
-        <v>6</v>
-      </c>
+      <c r="A223" s="2"/>
+      <c r="B223" s="2"/>
+      <c r="C223" s="2"/>
+      <c r="D223" s="2"/>
     </row>
     <row r="224" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A224" s="2" t="s">
-        <v>217</v>
-      </c>
-      <c r="B224" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C224" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D224" s="2" t="s">
-        <v>6</v>
-      </c>
+      <c r="A224" s="2"/>
+      <c r="B224" s="2"/>
+      <c r="C224" s="2"/>
+      <c r="D224" s="2"/>
     </row>
     <row r="225" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A225" s="2" t="s">
-        <v>218</v>
-      </c>
-      <c r="B225" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C225" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D225" s="2" t="s">
-        <v>6</v>
-      </c>
+      <c r="A225" s="2"/>
+      <c r="B225" s="2"/>
+      <c r="C225" s="2"/>
+      <c r="D225" s="2"/>
     </row>
     <row r="226" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A226" s="2" t="s">
-        <v>219</v>
-      </c>
-      <c r="B226" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="C226" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D226" s="2" t="s">
-        <v>168</v>
-      </c>
+      <c r="A226" s="2"/>
+      <c r="B226" s="2"/>
+      <c r="C226" s="2"/>
+      <c r="D226" s="2"/>
     </row>
     <row r="227" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A227" s="2" t="s">
-        <v>220</v>
-      </c>
-      <c r="B227" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C227" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D227" s="2" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="228" spans="1:4" ht="29" x14ac:dyDescent="0.35">
-      <c r="A228" s="2" t="s">
-        <v>221</v>
-      </c>
-      <c r="B228" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C228" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="D228" s="2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="229" spans="1:4" ht="29" x14ac:dyDescent="0.35">
-      <c r="A229" s="2" t="s">
-        <v>222</v>
-      </c>
-      <c r="B229" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C229" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="D229" s="2" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="230" spans="1:4" ht="29" x14ac:dyDescent="0.35">
-      <c r="A230" s="2" t="s">
-        <v>223</v>
-      </c>
-      <c r="B230" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="C230" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D230" s="2" t="s">
-        <v>168</v>
-      </c>
+      <c r="A227" s="2"/>
+      <c r="B227" s="2"/>
+      <c r="C227" s="2"/>
+      <c r="D227" s="2"/>
+    </row>
+    <row r="228" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A228" s="2"/>
+      <c r="B228" s="2"/>
+      <c r="C228" s="2"/>
+      <c r="D228" s="2"/>
+    </row>
+    <row r="229" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A229" s="2"/>
+      <c r="B229" s="2"/>
+      <c r="C229" s="2"/>
+      <c r="D229" s="2"/>
+    </row>
+    <row r="230" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A230" s="2"/>
+      <c r="B230" s="2"/>
+      <c r="C230" s="2"/>
+      <c r="D230" s="2"/>
     </row>
     <row r="231" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A231" s="2" t="s">
-        <v>224</v>
-      </c>
-      <c r="B231" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="C231" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D231" s="2" t="s">
-        <v>6</v>
-      </c>
+      <c r="A231" s="2"/>
+      <c r="B231" s="2"/>
+      <c r="C231" s="2"/>
+      <c r="D231" s="2"/>
     </row>
     <row r="232" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A232" s="2" t="s">
-        <v>225</v>
-      </c>
-      <c r="B232" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="C232" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D232" s="2" t="s">
-        <v>168</v>
-      </c>
+      <c r="A232" s="2"/>
+      <c r="B232" s="2"/>
+      <c r="C232" s="2"/>
+      <c r="D232" s="2"/>
     </row>
     <row r="233" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A233" s="2" t="s">
-        <v>226</v>
-      </c>
-      <c r="B233" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C233" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D233" s="2" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="234" spans="1:4" ht="29" x14ac:dyDescent="0.35">
-      <c r="A234" s="2" t="s">
-        <v>227</v>
-      </c>
-      <c r="B234" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C234" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="D234" s="2" t="s">
-        <v>6</v>
-      </c>
+      <c r="A233" s="2"/>
+      <c r="B233" s="2"/>
+      <c r="C233" s="2"/>
+      <c r="D233" s="2"/>
+    </row>
+    <row r="234" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A234" s="2"/>
+      <c r="B234" s="2"/>
+      <c r="C234" s="2"/>
+      <c r="D234" s="2"/>
     </row>
     <row r="235" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A235" s="2" t="s">
-        <v>228</v>
-      </c>
-      <c r="B235" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C235" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="D235" s="2" t="s">
-        <v>168</v>
-      </c>
+      <c r="A235" s="2"/>
+      <c r="B235" s="2"/>
+      <c r="C235" s="2"/>
+      <c r="D235" s="2"/>
     </row>
     <row r="236" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A236" s="2" t="s">
-        <v>229</v>
-      </c>
-      <c r="B236" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C236" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="D236" s="2" t="s">
-        <v>6</v>
-      </c>
+      <c r="A236" s="2"/>
+      <c r="B236" s="2"/>
+      <c r="C236" s="2"/>
+      <c r="D236" s="2"/>
     </row>
     <row r="237" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A237" s="2" t="s">
-        <v>230</v>
-      </c>
-      <c r="B237" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C237" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D237" s="2" t="s">
-        <v>168</v>
-      </c>
+      <c r="A237" s="2"/>
+      <c r="B237" s="2"/>
+      <c r="C237" s="2"/>
+      <c r="D237" s="2"/>
     </row>
     <row r="238" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A238" s="2" t="s">
-        <v>231</v>
-      </c>
-      <c r="B238" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C238" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D238" s="2" t="s">
-        <v>6</v>
-      </c>
+      <c r="A238" s="2"/>
+      <c r="B238" s="2"/>
+      <c r="C238" s="2"/>
+      <c r="D238" s="2"/>
+    </row>
+    <row r="239" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A239" s="2"/>
+      <c r="B239" s="2"/>
+      <c r="C239" s="2"/>
+      <c r="D239" s="2"/>
     </row>
     <row r="241" spans="10:11" x14ac:dyDescent="0.35">
       <c r="J241" s="1"/>
@@ -4785,7 +4639,7 @@
   </sheetData>
   <dataValidations count="1">
     <dataValidation type="list" showInputMessage="1" showErrorMessage="1" promptTitle="Variance Category" prompt="Income/Employment_x000a_Eligible Transactions_x000a_Credit/Housing_x000a_Assets/Reserves_x000a_Collateral_x000a_Debts/Liabilities_x000a_Matrix" sqref="B1" xr:uid="{29458ACD-77A7-493A-A755-0AC3373D25A9}">
-      <formula1>$B$2:$B$142</formula1>
+      <formula1>$B$2:$B$184</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>